<commit_message>
docs: Update Play Store release guide and generate release info Excel sheet with recent Q&A
</commit_message>
<xml_diff>
--- a/doc/google_play_release_info.xlsx
+++ b/doc/google_play_release_info.xlsx
@@ -490,10 +490,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="43.4" customWidth="1" min="1" max="1"/>
+    <col width="47.59999999999999" customWidth="1" min="1" max="1"/>
     <col width="85" customWidth="1" min="2" max="2"/>
     <col width="85" customWidth="1" min="3" max="3"/>
   </cols>
@@ -712,7 +712,7 @@
 ✨ 주요 기능
 1. AI 뉴스 키워드 브리핑 (Morning Briefing)
 - 관심 증시 및 뉴스 키워드를 지정하면 매일 아침 최신 국내 뉴스를 자동으로 모아줍니다.
-- 최신 Gemini AI가 복잡한 뉴스를 자연스러운 대화체로 깔끔하게 요약해 줍니다.
+- 최신 Gemini AI가 복잡한 뉴스를 자연스러운 대화체로 요약해 줍니다.
 - 음성 TTS 낭독 기능으로 출근 준비 중에도 편하게 뉴스를 들을 수 있습니다.
 2. 스마트 오디오 캡처 및 관리 (Audio Capture &amp; Management)
 - 고품질 녹음 및 전역 플레이어 지원
@@ -1182,12 +1182,122 @@
         </is>
       </c>
     </row>
+    <row r="42" ht="24" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>5. 개발자 프로필 및 계정 세부정보 선언 질문 정리 (신규)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>개발자 프로필 아이콘</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>ic_k_logo_3d.png 사용 유지 (512x512)</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>브랜드 엠블럼 디자인 시스템 통일성을 위해 그대로 사용</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>개발자 프로필 헤더 이미지</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>kdailyutil_developer_header.png (4096x2304 PNG)</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>딥차콜 배경 중앙에 오리지널 3D 육각 로고를 정확히 합성한 공식 헤더 파일 사용</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>개발자 공식 웹사이트 입력</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>https://kitwlsh.netlify.app/privacy-kdailyutil</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>도메인 메인 페이지가 비어 있을 경우, 에러 페이지 인식 회피를 위해 실제 작동하는 방침 주소 입력 팁</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>대한민국 추가 정보 선언</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>사업자/라이선스/대행사 정보 모두 공란(빈칸) 유지</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>KDailyUtil은 인앱 결제가 없는 100% 무료 앱이므로 통신판매업 및 사업자 신고 대상이 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>전화번호 본인 인증</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>국가 코드(+82)를 포함한 본인 번호 입력 후 문자 인증코드 입력 필수</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>인증 완료 후 [전화번호 확인됨](Verified) 마크가 떠야 게시 개요 에러가 완전 해결됨</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>구형 개발자 계정 혜택</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>2023년 11월 13일 이전 가입 계정 특혜 유지 (20인 테스트 조항 면제)</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>테스터 모집 없이 언제나 [프로덕션 (정식 출시)] 트랙으로 즉시 직행하여 배포 가능한 평생 특혜</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A24:C24"/>
     <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>